<commit_message>
Cierra Ridge limpio y prepara Huber clean
</commit_message>
<xml_diff>
--- a/Experimentos/grid_experimentos_radar.xlsx
+++ b/Experimentos/grid_experimentos_radar.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CONFIG_REFERENCIA" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CATALOGO_EXPERIMENTOS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="RESULTADOS_GRID" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="RUN_SUMMARY" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="RUN_ARTEFACTOS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_REFERENCIA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CATALOGO_EXPERIMENTOS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESULTADOS_GRID" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RUN_SUMMARY" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RUN_ARTEFACTOS" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001" forceFullCalc="1"/>
@@ -727,21 +727,21 @@
     <row r="13" ht="19.5" customHeight="1" s="27">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>• Horizonte sugerido: 1, 2, 3 y 4 semanas.</t>
+          <t>6) Cierre oficial E1 Ridge: E1_v5_clean queda como mejor Ridge limpio global y E1_v4_clean como referencia parsimoniosa.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="19.5" customHeight="1" s="27">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>• Pesos iniciales del documento: w1=30%, w2=25%, w3=30%, w4=15%; alpha=35%, beta=25%, gamma=25%, delta=10%, eta=5%.</t>
+          <t>7) El orden operativo del plan original continua con E2 Huber antes de E3 Random Forest y E4 XGBoost / LightGBM.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="19.5" customHeight="1" s="27">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>• Puedes cambiar los pesos en 'CONFIG_REFERENCIA' y todas las fórmulas se actualizarán.</t>
+          <t>8) No se continua automaticamente con E1_v6+; Ridge queda cerrado como baseline lineal regularizado principal.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="G2" s="57" t="inlineStr">
         <is>
-          <t>Buen baseline para señal real e interpretabilidad</t>
+          <t>Ridge cerrado como rama principal: E1_v5_clean mejor global por L_total_Radar; E1_v4_clean referencia parsimoniosa. No continuar automaticamente con E1_v6+.</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="G3" s="57" t="inlineStr">
         <is>
-          <t>Útil si hay ruido, shocks y colas</t>
+          <t>Siguiente familia del plan original: Huber con el mismo marco de evaluacion temporal, tuning interno temporal y perdida Radar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cierra E2 y prepara familia E3
</commit_message>
<xml_diff>
--- a/Experimentos/grid_experimentos_radar.xlsx
+++ b/Experimentos/grid_experimentos_radar.xlsx
@@ -734,18 +734,24 @@
     <row r="14" ht="19.5" customHeight="1" s="27">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>7) El orden operativo del plan original continua con E2 Huber antes de E3 Random Forest y E4 XGBoost / LightGBM.</t>
+          <t>7) Cierre oficial E2 Huber: E2_v3_clean gana internamente, E2_v2_clean descarta convergencia como causa principal y la familia queda cerrada.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="19.5" customHeight="1" s="27">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>8) No se continua automaticamente con E1_v6+; Ridge queda cerrado como baseline lineal regularizado principal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="19.5" customHeight="1" s="27"/>
+          <t>8) E2_v4_clean queda cancelada por decision metodologica explicita y no se ejecuta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="19.5" customHeight="1" s="27">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9) Siguiente prioridad operativa: E3 Random Forest con el mismo marco temporal limpio; E4 XGBoost y E5 CatBoost quedan como continuidad.</t>
+        </is>
+      </c>
+    </row>
     <row r="17" ht="19.5" customHeight="1" s="27">
       <c r="A17" s="30" t="inlineStr">
         <is>
@@ -1261,7 +1267,7 @@
       </c>
       <c r="G3" s="57" t="inlineStr">
         <is>
-          <t>Siguiente familia del plan original: Huber con el mismo marco de evaluacion temporal, tuning interno temporal y perdida Radar.</t>
+          <t>Familia cerrada bajo esquema limpio temporal: E2_v3_clean gana internamente, E2_v2_clean descarta convergencia como explicacion principal y E2_v4_clean se cancela por decision metodologica. No competitiva frente a E1_v5_clean.</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1304,7 @@
       </c>
       <c r="G4" s="57" t="inlineStr">
         <is>
-          <t>Puede captar interacciones sin mucho tuning</t>
+          <t>Siguiente prioridad operativa: Random Forest clean con el mismo marco temporal. Referencia principal E1_v5_clean; referencias secundarias E1_v4_clean y E2_v3_clean.</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1341,7 @@
       </c>
       <c r="G5" s="57" t="inlineStr">
         <is>
-          <t>Muy buen candidato para desempeño</t>
+          <t>Continuidad natural de E3: XGBoost / LightGBM con la misma arquitectura limpia por familias.</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1378,7 @@
       </c>
       <c r="G6" s="57" t="inlineStr">
         <is>
-          <t>Suele funcionar bien con estructura tabular</t>
+          <t>Continuidad de boosting: CatBoost con el mismo marco temporal y comparaciones contra E1/E3.</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AK161"/>
+  <dimension ref="A1:AK173"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="26" min="1" max="1"/>
@@ -14817,6 +14823,1890 @@
       <c r="AK161" s="49" t="inlineStr">
         <is>
           <t>2026-03-21 10:54:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="15" customHeight="1" s="27">
+      <c r="A162" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:00:29</t>
+        </is>
+      </c>
+      <c r="B162" s="49" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C162" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D162" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E162" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F162" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G162" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H162" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4, 5, 6]</t>
+        </is>
+      </c>
+      <c r="I162" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J162" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K162" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L162" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M162" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N162" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 83, "feature_mode": "corr", "horizon": 1, "initial_train_size": 40, "lags": [1, 2, 3, 4, 5, 6], "model": "huber_tscv", "model_params": {"inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [1000], "tol": [0.0001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 26, "rows_modeling": 66, "selected_feature_count_avg": 30.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O162" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P162" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q162" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R162" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S162" s="52" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T162" s="53" t="n">
+        <v>0.184685768753275</v>
+      </c>
+      <c r="U162" s="53" t="n">
+        <v>0.2307692307692307</v>
+      </c>
+      <c r="V162" s="53" t="n">
+        <v>0.1666666666666666</v>
+      </c>
+      <c r="W162" s="53" t="n">
+        <v>0.6538461538461539</v>
+      </c>
+      <c r="X162" s="54" t="n">
+        <v>0.06881508264217079</v>
+      </c>
+      <c r="Y162" s="53" t="n">
+        <v>0.1136342110145291</v>
+      </c>
+      <c r="Z162" s="53" t="n">
+        <v>0.1492880502016995</v>
+      </c>
+      <c r="AA162" s="55" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="AB162" s="55" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="AC162" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD162" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE162" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF162" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG162" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029</t>
+        </is>
+      </c>
+      <c r="AH162" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI162" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ162" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK162" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:00:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="15" customHeight="1" s="27">
+      <c r="A163" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:00:29</t>
+        </is>
+      </c>
+      <c r="B163" s="49" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C163" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D163" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E163" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F163" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="G163" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H163" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4, 5, 6]</t>
+        </is>
+      </c>
+      <c r="I163" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J163" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K163" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L163" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M163" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N163" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 83, "feature_mode": "corr", "horizon": 2, "initial_train_size": 40, "lags": [1, 2, 3, 4, 5, 6], "model": "huber_tscv", "model_params": {"inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [1000], "tol": [0.0001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 25, "rows_modeling": 65, "selected_feature_count_avg": 30.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O163" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P163" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q163" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R163" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S163" s="52" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="T163" s="53" t="n">
+        <v>0.198125454400369</v>
+      </c>
+      <c r="U163" s="53" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="V163" s="53" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="W163" s="53" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="X163" s="54" t="n">
+        <v>0.0870859772600323</v>
+      </c>
+      <c r="Y163" s="53" t="n">
+        <v>0.1219034354658784</v>
+      </c>
+      <c r="Z163" s="53" t="n">
+        <v>0.1466092520563559</v>
+      </c>
+      <c r="AA163" s="55" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AB163" s="55" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AC163" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD163" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE163" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF163" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG163" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029</t>
+        </is>
+      </c>
+      <c r="AH163" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI163" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ163" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK163" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:00:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="15" customHeight="1" s="27">
+      <c r="A164" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:00:29</t>
+        </is>
+      </c>
+      <c r="B164" s="49" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C164" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D164" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E164" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F164" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="G164" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H164" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4, 5, 6]</t>
+        </is>
+      </c>
+      <c r="I164" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J164" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K164" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L164" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M164" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N164" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 83, "feature_mode": "corr", "horizon": 3, "initial_train_size": 40, "lags": [1, 2, 3, 4, 5, 6], "model": "huber_tscv", "model_params": {"inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [1000], "tol": [0.0001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 24, "rows_modeling": 64, "selected_feature_count_avg": 30.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O164" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P164" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q164" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R164" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S164" s="52" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T164" s="53" t="n">
+        <v>0.258896465891488</v>
+      </c>
+      <c r="U164" s="53" t="n">
+        <v>0.2916666666666666</v>
+      </c>
+      <c r="V164" s="53" t="n">
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="W164" s="53" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="X164" s="54" t="n">
+        <v>0.08394549255496986</v>
+      </c>
+      <c r="Y164" s="53" t="n">
+        <v>0.1592948706044114</v>
+      </c>
+      <c r="Z164" s="53" t="n">
+        <v>0.2059121290091017</v>
+      </c>
+      <c r="AA164" s="55" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="AB164" s="55" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="AC164" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD164" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE164" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF164" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG164" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029</t>
+        </is>
+      </c>
+      <c r="AH164" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI164" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ164" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK164" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:00:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="15" customHeight="1" s="27">
+      <c r="A165" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:00:29</t>
+        </is>
+      </c>
+      <c r="B165" s="49" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C165" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D165" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E165" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F165" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="G165" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H165" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4, 5, 6]</t>
+        </is>
+      </c>
+      <c r="I165" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J165" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K165" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L165" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M165" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N165" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 83, "feature_mode": "corr", "horizon": 4, "initial_train_size": 40, "lags": [1, 2, 3, 4, 5, 6], "model": "huber_tscv", "model_params": {"inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [1000], "tol": [0.0001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 23, "rows_modeling": 63, "selected_feature_count_avg": 30.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O165" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P165" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q165" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R165" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S165" s="52" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="T165" s="53" t="n">
+        <v>0.3118545795245171</v>
+      </c>
+      <c r="U165" s="53" t="n">
+        <v>0.4782608695652174</v>
+      </c>
+      <c r="V165" s="53" t="n">
+        <v>0.4444444444444444</v>
+      </c>
+      <c r="W165" s="53" t="n">
+        <v>0.7391304347826086</v>
+      </c>
+      <c r="X165" s="54" t="n">
+        <v>0.06206077122213859</v>
+      </c>
+      <c r="Y165" s="53" t="n">
+        <v>0.1918791541695755</v>
+      </c>
+      <c r="Z165" s="53" t="n">
+        <v>0.2633428327259931</v>
+      </c>
+      <c r="AA165" s="55" t="n">
+        <v>0.5217391304347826</v>
+      </c>
+      <c r="AB165" s="55" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="AC165" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD165" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE165" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF165" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG165" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029</t>
+        </is>
+      </c>
+      <c r="AH165" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI165" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ165" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK165" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:00:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="15" customHeight="1" s="27">
+      <c r="A166" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:41:01</t>
+        </is>
+      </c>
+      <c r="B166" s="49" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C166" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D166" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E166" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F166" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G166" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H166" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4, 5, 6]</t>
+        </is>
+      </c>
+      <c r="I166" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J166" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K166" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L166" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M166" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N166" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 83, "feature_mode": "corr", "horizon": 1, "initial_train_size": 40, "lags": [1, 2, 3, 4, 5, 6], "model": "huber_tscv", "model_params": {"hypothesis_note": "control_de_convergencia", "inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [5000], "tol": [0.0001, 0.001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 26, "rows_modeling": 66, "selected_feature_count_avg": 30.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O166" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P166" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q166" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R166" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S166" s="52" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T166" s="53" t="n">
+        <v>0.1848095621248963</v>
+      </c>
+      <c r="U166" s="53" t="n">
+        <v>0.2307692307692307</v>
+      </c>
+      <c r="V166" s="53" t="n">
+        <v>0.1666666666666666</v>
+      </c>
+      <c r="W166" s="53" t="n">
+        <v>0.6538461538461539</v>
+      </c>
+      <c r="X166" s="54" t="n">
+        <v>0.06882808094619103</v>
+      </c>
+      <c r="Y166" s="53" t="n">
+        <v>0.1137103791037543</v>
+      </c>
+      <c r="Z166" s="53" t="n">
+        <v>0.1491199728508273</v>
+      </c>
+      <c r="AA166" s="55" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="AB166" s="55" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="AC166" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD166" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | hipotesis=control_de_convergencia | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE166" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF166" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG166" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101</t>
+        </is>
+      </c>
+      <c r="AH166" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI166" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ166" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK166" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:41:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="15" customHeight="1" s="27">
+      <c r="A167" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:41:01</t>
+        </is>
+      </c>
+      <c r="B167" s="49" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C167" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D167" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E167" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F167" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="G167" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H167" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4, 5, 6]</t>
+        </is>
+      </c>
+      <c r="I167" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J167" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K167" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L167" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M167" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N167" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 83, "feature_mode": "corr", "horizon": 2, "initial_train_size": 40, "lags": [1, 2, 3, 4, 5, 6], "model": "huber_tscv", "model_params": {"hypothesis_note": "control_de_convergencia", "inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [5000], "tol": [0.0001, 0.001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 25, "rows_modeling": 65, "selected_feature_count_avg": 30.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O167" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P167" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q167" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R167" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S167" s="52" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="T167" s="53" t="n">
+        <v>0.198125454400369</v>
+      </c>
+      <c r="U167" s="53" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="V167" s="53" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="W167" s="53" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="X167" s="54" t="n">
+        <v>0.0870859772600323</v>
+      </c>
+      <c r="Y167" s="53" t="n">
+        <v>0.1219034354658784</v>
+      </c>
+      <c r="Z167" s="53" t="n">
+        <v>0.1466092520563559</v>
+      </c>
+      <c r="AA167" s="55" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AB167" s="55" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AC167" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD167" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | hipotesis=control_de_convergencia | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE167" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF167" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG167" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101</t>
+        </is>
+      </c>
+      <c r="AH167" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI167" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ167" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK167" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:41:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="15" customHeight="1" s="27">
+      <c r="A168" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:41:01</t>
+        </is>
+      </c>
+      <c r="B168" s="49" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C168" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D168" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E168" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F168" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="G168" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H168" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4, 5, 6]</t>
+        </is>
+      </c>
+      <c r="I168" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J168" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K168" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L168" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M168" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N168" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 83, "feature_mode": "corr", "horizon": 3, "initial_train_size": 40, "lags": [1, 2, 3, 4, 5, 6], "model": "huber_tscv", "model_params": {"hypothesis_note": "control_de_convergencia", "inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [5000], "tol": [0.0001, 0.001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 24, "rows_modeling": 64, "selected_feature_count_avg": 30.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O168" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P168" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q168" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R168" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S168" s="52" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T168" s="53" t="n">
+        <v>0.258896465891488</v>
+      </c>
+      <c r="U168" s="53" t="n">
+        <v>0.2916666666666666</v>
+      </c>
+      <c r="V168" s="53" t="n">
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="W168" s="53" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="X168" s="54" t="n">
+        <v>0.08394549255496986</v>
+      </c>
+      <c r="Y168" s="53" t="n">
+        <v>0.1592948706044114</v>
+      </c>
+      <c r="Z168" s="53" t="n">
+        <v>0.2059121290091017</v>
+      </c>
+      <c r="AA168" s="55" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="AB168" s="55" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="AC168" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD168" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | hipotesis=control_de_convergencia | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE168" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF168" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG168" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101</t>
+        </is>
+      </c>
+      <c r="AH168" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI168" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ168" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK168" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:41:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="15" customHeight="1" s="27">
+      <c r="A169" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:41:01</t>
+        </is>
+      </c>
+      <c r="B169" s="49" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C169" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D169" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E169" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F169" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="G169" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H169" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4, 5, 6]</t>
+        </is>
+      </c>
+      <c r="I169" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J169" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K169" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L169" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M169" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N169" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 83, "feature_mode": "corr", "horizon": 4, "initial_train_size": 40, "lags": [1, 2, 3, 4, 5, 6], "model": "huber_tscv", "model_params": {"hypothesis_note": "control_de_convergencia", "inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [5000], "tol": [0.0001, 0.001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 23, "rows_modeling": 63, "selected_feature_count_avg": 30.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O169" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P169" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q169" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R169" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S169" s="52" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="T169" s="53" t="n">
+        <v>0.3118545795245171</v>
+      </c>
+      <c r="U169" s="53" t="n">
+        <v>0.4782608695652174</v>
+      </c>
+      <c r="V169" s="53" t="n">
+        <v>0.4444444444444444</v>
+      </c>
+      <c r="W169" s="53" t="n">
+        <v>0.7391304347826086</v>
+      </c>
+      <c r="X169" s="54" t="n">
+        <v>0.06206077122213859</v>
+      </c>
+      <c r="Y169" s="53" t="n">
+        <v>0.1918791541695755</v>
+      </c>
+      <c r="Z169" s="53" t="n">
+        <v>0.2633428327259931</v>
+      </c>
+      <c r="AA169" s="55" t="n">
+        <v>0.5217391304347826</v>
+      </c>
+      <c r="AB169" s="55" t="n">
+        <v>0.5555555555555556</v>
+      </c>
+      <c r="AC169" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD169" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | hipotesis=control_de_convergencia | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE169" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF169" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG169" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101</t>
+        </is>
+      </c>
+      <c r="AH169" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI169" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ169" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK169" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:41:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="15" customHeight="1" s="27">
+      <c r="A170" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:12:13</t>
+        </is>
+      </c>
+      <c r="B170" s="49" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C170" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D170" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E170" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F170" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G170" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H170" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="I170" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J170" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K170" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L170" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M170" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N170" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 59, "feature_mode": "corr", "horizon": 1, "initial_train_size": 40, "lags": [1, 2, 3, 4], "model": "huber_tscv", "model_params": {"hypothesis_note": "prueba_sin_memoria_larga", "inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [1000], "tol": [0.0001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 28, "rows_modeling": 68, "selected_feature_count_avg": 21.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O170" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P170" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q170" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R170" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S170" s="52" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T170" s="53" t="n">
+        <v>0.1945968068018527</v>
+      </c>
+      <c r="U170" s="53" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="V170" s="53" t="n">
+        <v>0.1538461538461539</v>
+      </c>
+      <c r="W170" s="53" t="n">
+        <v>0.6785714285714286</v>
+      </c>
+      <c r="X170" s="54" t="n">
+        <v>0.07107826910979893</v>
+      </c>
+      <c r="Y170" s="53" t="n">
+        <v>0.1197323148185621</v>
+      </c>
+      <c r="Z170" s="53" t="n">
+        <v>0.1499850473896837</v>
+      </c>
+      <c r="AA170" s="55" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AB170" s="55" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="AC170" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD170" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | hipotesis=prueba_sin_memoria_larga | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE170" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF170" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG170" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213</t>
+        </is>
+      </c>
+      <c r="AH170" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI170" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ170" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK170" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:12:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="15" customHeight="1" s="27">
+      <c r="A171" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:12:13</t>
+        </is>
+      </c>
+      <c r="B171" s="49" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C171" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D171" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E171" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F171" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="G171" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H171" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="I171" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J171" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K171" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L171" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M171" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N171" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 59, "feature_mode": "corr", "horizon": 2, "initial_train_size": 40, "lags": [1, 2, 3, 4], "model": "huber_tscv", "model_params": {"hypothesis_note": "prueba_sin_memoria_larga", "inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [1000], "tol": [0.0001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 27, "rows_modeling": 67, "selected_feature_count_avg": 21.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O171" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P171" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q171" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R171" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S171" s="52" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="T171" s="53" t="n">
+        <v>0.1845910273692062</v>
+      </c>
+      <c r="U171" s="53" t="n">
+        <v>0.3333333333333334</v>
+      </c>
+      <c r="V171" s="53" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="W171" s="53" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="X171" s="54" t="n">
+        <v>0.06927671489480554</v>
+      </c>
+      <c r="Y171" s="53" t="n">
+        <v>0.1135759181503753</v>
+      </c>
+      <c r="Z171" s="53" t="n">
+        <v>0.1479713958144309</v>
+      </c>
+      <c r="AA171" s="55" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="AB171" s="55" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AC171" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD171" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | hipotesis=prueba_sin_memoria_larga | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE171" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF171" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG171" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213</t>
+        </is>
+      </c>
+      <c r="AH171" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI171" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ171" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK171" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:12:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="15" customHeight="1" s="27">
+      <c r="A172" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:12:13</t>
+        </is>
+      </c>
+      <c r="B172" s="49" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C172" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D172" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E172" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F172" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="G172" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H172" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="I172" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J172" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K172" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L172" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M172" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N172" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 59, "feature_mode": "corr", "horizon": 3, "initial_train_size": 40, "lags": [1, 2, 3, 4], "model": "huber_tscv", "model_params": {"hypothesis_note": "prueba_sin_memoria_larga", "inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [1000], "tol": [0.0001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 26, "rows_modeling": 66, "selected_feature_count_avg": 21.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O172" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P172" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q172" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R172" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S172" s="52" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T172" s="53" t="n">
+        <v>0.2306409358773327</v>
+      </c>
+      <c r="U172" s="53" t="n">
+        <v>0.3461538461538461</v>
+      </c>
+      <c r="V172" s="53" t="n">
+        <v>0.4166666666666666</v>
+      </c>
+      <c r="W172" s="53" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="X172" s="54" t="n">
+        <v>0.1091211444209661</v>
+      </c>
+      <c r="Y172" s="53" t="n">
+        <v>0.1419096931669162</v>
+      </c>
+      <c r="Z172" s="53" t="n">
+        <v>0.1631289658990064</v>
+      </c>
+      <c r="AA172" s="55" t="n">
+        <v>0.6538461538461539</v>
+      </c>
+      <c r="AB172" s="55" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="AC172" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD172" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | hipotesis=prueba_sin_memoria_larga | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE172" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF172" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG172" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213</t>
+        </is>
+      </c>
+      <c r="AH172" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI172" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ172" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK172" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:12:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="15" customHeight="1" s="27">
+      <c r="A173" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:12:13</t>
+        </is>
+      </c>
+      <c r="B173" s="49" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C173" s="50" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D173" s="50" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E173" s="50" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="F173" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="G173" s="49" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="H173" s="50" t="inlineStr">
+        <is>
+          <t>y_t + lags [1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="I173" s="50" t="inlineStr">
+        <is>
+          <t>sentimiento_medios, v5_agua_neto, v5_alumbrado_neto, v5_americo_neto, v5_basura_neto, v5_corrupcion_neto, v5_delitos_neto, v5_morena_neto, v5_obras_neto, v5_prevencion_neto, v5_vialidad_neto</t>
+        </is>
+      </c>
+      <c r="J173" s="50" t="inlineStr">
+        <is>
+          <t>standard_scaler</t>
+        </is>
+      </c>
+      <c r="K173" s="50" t="inlineStr">
+        <is>
+          <t>corr</t>
+        </is>
+      </c>
+      <c r="L173" s="50" t="inlineStr">
+        <is>
+          <t>walk-forward_expanding</t>
+        </is>
+      </c>
+      <c r="M173" s="49" t="inlineStr">
+        <is>
+          <t>2024-10-14 a 2026-03-02</t>
+        </is>
+      </c>
+      <c r="N173" s="49" t="inlineStr">
+        <is>
+          <t>{"feature_candidates": 59, "feature_mode": "corr", "horizon": 4, "initial_train_size": 40, "lags": [1, 2, 3, 4], "model": "huber_tscv", "model_params": {"hypothesis_note": "prueba_sin_memoria_larga", "inner_splits": 3, "param_grid": {"alpha": [1e-06, 9.999999999999999e-06, 0.0001, 0.001, 0.01, 0.1], "epsilon": [1.1, 1.2, 1.35, 1.5, 1.75, 2.0], "max_iter": [1000], "tol": [0.0001]}, "transform_mode": "standard", "tuning_metric": "mae", "winsor_lower_quantile": 0.05, "winsor_upper_quantile": 0.95}, "rows_eval": 25, "rows_modeling": 65, "selected_feature_count_avg": 21.0, "target_mode": "nivel", "transform_mode": "standard"}</t>
+        </is>
+      </c>
+      <c r="O173" s="51" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P173" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q173" s="51" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="R173" s="51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S173" s="52" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="T173" s="53" t="n">
+        <v>0.2331120640375527</v>
+      </c>
+      <c r="U173" s="53" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="V173" s="53" t="n">
+        <v>0.09999999999999998</v>
+      </c>
+      <c r="W173" s="53" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="X173" s="54" t="n">
+        <v>0.03698838336197151</v>
+      </c>
+      <c r="Y173" s="53" t="n">
+        <v>0.1434301389527392</v>
+      </c>
+      <c r="Z173" s="53" t="n">
+        <v>0.167126942327339</v>
+      </c>
+      <c r="AA173" s="55" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="AB173" s="55" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC173" s="49" t="inlineStr">
+        <is>
+          <t>corrido</t>
+        </is>
+      </c>
+      <c r="AD173" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning temporal interno | hipotesis=prueba_sin_memoria_larga | metric=mae | inner_splits=3</t>
+        </is>
+      </c>
+      <c r="AE173" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AF173" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AG173" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213</t>
+        </is>
+      </c>
+      <c r="AH173" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="AI173" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="AJ173" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="AK173" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:12:13</t>
         </is>
       </c>
     </row>
@@ -14885,7 +16775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:W106"/>
+  <dimension ref="A1:W109"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="26" min="1" max="1"/>
@@ -21634,6 +23524,273 @@
       <c r="W106" s="49" t="inlineStr">
         <is>
           <t>2026-03-21 10:54:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="15" customHeight="1" s="27">
+      <c r="A107" s="49" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="B107" s="57" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C107" s="57" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="D107" s="57" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E107" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="F107" s="54" t="n">
+        <v>0.3019073236793116</v>
+      </c>
+      <c r="G107" s="53" t="n"/>
+      <c r="H107" s="58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I107" s="54" t="n">
+        <v>0.3019073236793116</v>
+      </c>
+      <c r="J107" s="54" t="n">
+        <v>0.1466779178135986</v>
+      </c>
+      <c r="K107" s="54" t="n">
+        <v>0.1912880659982875</v>
+      </c>
+      <c r="L107" s="51" t="n">
+        <v>0.6298258082497213</v>
+      </c>
+      <c r="M107" s="51" t="n">
+        <v>0.7267676767676767</v>
+      </c>
+      <c r="N107" s="49" t="n"/>
+      <c r="O107" s="57" t="n"/>
+      <c r="P107" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning interno TimeSeriesSplit | metric=mae | L_total_Radar=0.301907</t>
+        </is>
+      </c>
+      <c r="Q107" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="R107" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="S107" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029</t>
+        </is>
+      </c>
+      <c r="T107" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="U107" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="V107" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="W107" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:00:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="15" customHeight="1" s="27">
+      <c r="A108" s="49" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="B108" s="57" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C108" s="57" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="D108" s="57" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E108" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="F108" s="54" t="n">
+        <v>0.3019203219833318</v>
+      </c>
+      <c r="G108" s="53" t="n"/>
+      <c r="H108" s="58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I108" s="54" t="n">
+        <v>0.3019203219833318</v>
+      </c>
+      <c r="J108" s="54" t="n">
+        <v>0.1466969598359049</v>
+      </c>
+      <c r="K108" s="54" t="n">
+        <v>0.1912460466605695</v>
+      </c>
+      <c r="L108" s="51" t="n">
+        <v>0.6298258082497213</v>
+      </c>
+      <c r="M108" s="51" t="n">
+        <v>0.7267676767676767</v>
+      </c>
+      <c r="N108" s="49" t="n"/>
+      <c r="O108" s="57" t="n"/>
+      <c r="P108" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning interno TimeSeriesSplit | hipotesis=control_de_convergencia | metric=mae | L_total_Radar=0.301920</t>
+        </is>
+      </c>
+      <c r="Q108" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="R108" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="S108" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101</t>
+        </is>
+      </c>
+      <c r="T108" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="U108" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="V108" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="W108" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:41:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="15" customHeight="1" s="27">
+      <c r="A109" s="49" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="B109" s="57" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="C109" s="57" t="inlineStr">
+        <is>
+          <t>huber_tscv</t>
+        </is>
+      </c>
+      <c r="D109" s="57" t="inlineStr">
+        <is>
+          <t>robusto</t>
+        </is>
+      </c>
+      <c r="E109" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="F109" s="54" t="n">
+        <v>0.2864645117875421</v>
+      </c>
+      <c r="G109" s="53" t="n"/>
+      <c r="H109" s="58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I109" s="54" t="n">
+        <v>0.2864645117875421</v>
+      </c>
+      <c r="J109" s="54" t="n">
+        <v>0.1296620162721482</v>
+      </c>
+      <c r="K109" s="54" t="n">
+        <v>0.157053087857615</v>
+      </c>
+      <c r="L109" s="51" t="n">
+        <v>0.707628205128205</v>
+      </c>
+      <c r="M109" s="51" t="n">
+        <v>0.7698717948717949</v>
+      </c>
+      <c r="N109" s="49" t="n"/>
+      <c r="O109" s="57" t="n"/>
+      <c r="P109" s="49" t="inlineStr">
+        <is>
+          <t>Huber limpio con tuning interno TimeSeriesSplit | hipotesis=prueba_sin_memoria_larga | metric=mae | L_total_Radar=0.286465</t>
+        </is>
+      </c>
+      <c r="Q109" s="49" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="R109" s="49" t="inlineStr">
+        <is>
+          <t>Scripts/Modeling/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="S109" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213</t>
+        </is>
+      </c>
+      <c r="T109" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="U109" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="V109" s="49" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="W109" s="49" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:12:13</t>
         </is>
       </c>
     </row>
@@ -21677,7 +23834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="26" min="1" max="6"/>
@@ -24320,6 +26477,1745 @@
         </is>
       </c>
     </row>
+    <row r="73" ht="15" customHeight="1" s="27">
+      <c r="A73" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B73" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C73" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D73" s="61" t="inlineStr">
+        <is>
+          <t>script_snapshot</t>
+        </is>
+      </c>
+      <c r="E73" s="61" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="F73" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="G73" s="61" t="inlineStr">
+        <is>
+          <t>Copia del script ejecutado para reproducibilidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="15" customHeight="1" s="27">
+      <c r="A74" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B74" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C74" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D74" s="61" t="inlineStr">
+        <is>
+          <t>parametros</t>
+        </is>
+      </c>
+      <c r="E74" s="61" t="inlineStr">
+        <is>
+          <t>parametros_run.json</t>
+        </is>
+      </c>
+      <c r="F74" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="G74" s="61" t="inlineStr">
+        <is>
+          <t>Parametros del experimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="15" customHeight="1" s="27">
+      <c r="A75" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B75" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C75" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D75" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E75" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h1.csv</t>
+        </is>
+      </c>
+      <c r="F75" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/features_seleccionadas_h1.csv</t>
+        </is>
+      </c>
+      <c r="G75" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="15" customHeight="1" s="27">
+      <c r="A76" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B76" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C76" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D76" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E76" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h2.csv</t>
+        </is>
+      </c>
+      <c r="F76" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/features_seleccionadas_h2.csv</t>
+        </is>
+      </c>
+      <c r="G76" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="15" customHeight="1" s="27">
+      <c r="A77" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B77" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C77" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D77" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E77" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h3.csv</t>
+        </is>
+      </c>
+      <c r="F77" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/features_seleccionadas_h3.csv</t>
+        </is>
+      </c>
+      <c r="G77" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="15" customHeight="1" s="27">
+      <c r="A78" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B78" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C78" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D78" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E78" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h4.csv</t>
+        </is>
+      </c>
+      <c r="F78" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/features_seleccionadas_h4.csv</t>
+        </is>
+      </c>
+      <c r="G78" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="15" customHeight="1" s="27">
+      <c r="A79" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B79" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C79" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D79" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E79" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h1.csv</t>
+        </is>
+      </c>
+      <c r="F79" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/predicciones_h1.csv</t>
+        </is>
+      </c>
+      <c r="G79" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="15" customHeight="1" s="27">
+      <c r="A80" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B80" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C80" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D80" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E80" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h2.csv</t>
+        </is>
+      </c>
+      <c r="F80" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/predicciones_h2.csv</t>
+        </is>
+      </c>
+      <c r="G80" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="15" customHeight="1" s="27">
+      <c r="A81" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B81" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C81" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D81" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E81" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h3.csv</t>
+        </is>
+      </c>
+      <c r="F81" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/predicciones_h3.csv</t>
+        </is>
+      </c>
+      <c r="G81" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="15" customHeight="1" s="27">
+      <c r="A82" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B82" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C82" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D82" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E82" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h4.csv</t>
+        </is>
+      </c>
+      <c r="F82" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/predicciones_h4.csv</t>
+        </is>
+      </c>
+      <c r="G82" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15" customHeight="1" s="27">
+      <c r="A83" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B83" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C83" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D83" s="61" t="inlineStr">
+        <is>
+          <t>resumen</t>
+        </is>
+      </c>
+      <c r="E83" s="61" t="inlineStr">
+        <is>
+          <t>resumen_modeling_horizontes.json</t>
+        </is>
+      </c>
+      <c r="F83" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/resumen_modeling_horizontes.json</t>
+        </is>
+      </c>
+      <c r="G83" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de tamanos y seleccion de features por horizonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="15" customHeight="1" s="27">
+      <c r="A84" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B84" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C84" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D84" s="61" t="inlineStr">
+        <is>
+          <t>tuning</t>
+        </is>
+      </c>
+      <c r="E84" s="61" t="inlineStr">
+        <is>
+          <t>huber_tuning_horizontes.json</t>
+        </is>
+      </c>
+      <c r="F84" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/huber_tuning_horizontes.json</t>
+        </is>
+      </c>
+      <c r="G84" s="61" t="inlineStr">
+        <is>
+          <t>Mejores hiperparametros Huber por fold externo y resumen por horizonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="15" customHeight="1" s="27">
+      <c r="A85" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B85" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C85" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D85" s="61" t="inlineStr">
+        <is>
+          <t>comparacion</t>
+        </is>
+      </c>
+      <c r="E85" s="61" t="inlineStr">
+        <is>
+          <t>comparacion_vs_E1_v5_clean.json</t>
+        </is>
+      </c>
+      <c r="F85" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/comparacion_vs_E1_v5_clean.json</t>
+        </is>
+      </c>
+      <c r="G85" s="61" t="inlineStr">
+        <is>
+          <t>Comparacion de la corrida clean contra E1_v5_clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15" customHeight="1" s="27">
+      <c r="A86" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B86" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C86" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D86" s="61" t="inlineStr">
+        <is>
+          <t>metricas</t>
+        </is>
+      </c>
+      <c r="E86" s="61" t="inlineStr">
+        <is>
+          <t>metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="F86" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="G86" s="61" t="inlineStr">
+        <is>
+          <t>Resumen estructurado por horizonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="15" customHeight="1" s="27">
+      <c r="A87" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 05:15:03</t>
+        </is>
+      </c>
+      <c r="B87" s="61" t="inlineStr">
+        <is>
+          <t>E2_v1_clean</t>
+        </is>
+      </c>
+      <c r="C87" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D87" s="61" t="inlineStr">
+        <is>
+          <t>metadata</t>
+        </is>
+      </c>
+      <c r="E87" s="61" t="inlineStr">
+        <is>
+          <t>metadata_run.json</t>
+        </is>
+      </c>
+      <c r="F87" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v1_clean_20260323_050029/metadata_run.json</t>
+        </is>
+      </c>
+      <c r="G87" s="61" t="inlineStr">
+        <is>
+          <t>Metadata base del run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="15" customHeight="1" s="27">
+      <c r="A88" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B88" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C88" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D88" s="61" t="inlineStr">
+        <is>
+          <t>script_snapshot</t>
+        </is>
+      </c>
+      <c r="E88" s="61" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="F88" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="G88" s="61" t="inlineStr">
+        <is>
+          <t>Copia del script ejecutado para reproducibilidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="15" customHeight="1" s="27">
+      <c r="A89" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B89" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C89" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D89" s="61" t="inlineStr">
+        <is>
+          <t>parametros</t>
+        </is>
+      </c>
+      <c r="E89" s="61" t="inlineStr">
+        <is>
+          <t>parametros_run.json</t>
+        </is>
+      </c>
+      <c r="F89" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="G89" s="61" t="inlineStr">
+        <is>
+          <t>Parametros del experimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="15" customHeight="1" s="27">
+      <c r="A90" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B90" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C90" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D90" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E90" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h1.csv</t>
+        </is>
+      </c>
+      <c r="F90" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/features_seleccionadas_h1.csv</t>
+        </is>
+      </c>
+      <c r="G90" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="15" customHeight="1" s="27">
+      <c r="A91" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B91" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C91" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D91" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E91" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h2.csv</t>
+        </is>
+      </c>
+      <c r="F91" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/features_seleccionadas_h2.csv</t>
+        </is>
+      </c>
+      <c r="G91" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="15" customHeight="1" s="27">
+      <c r="A92" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B92" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C92" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D92" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E92" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h3.csv</t>
+        </is>
+      </c>
+      <c r="F92" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/features_seleccionadas_h3.csv</t>
+        </is>
+      </c>
+      <c r="G92" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="15" customHeight="1" s="27">
+      <c r="A93" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B93" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C93" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D93" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E93" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h4.csv</t>
+        </is>
+      </c>
+      <c r="F93" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/features_seleccionadas_h4.csv</t>
+        </is>
+      </c>
+      <c r="G93" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="15" customHeight="1" s="27">
+      <c r="A94" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B94" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C94" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D94" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E94" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h1.csv</t>
+        </is>
+      </c>
+      <c r="F94" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/predicciones_h1.csv</t>
+        </is>
+      </c>
+      <c r="G94" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="15" customHeight="1" s="27">
+      <c r="A95" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B95" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C95" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D95" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E95" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h2.csv</t>
+        </is>
+      </c>
+      <c r="F95" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/predicciones_h2.csv</t>
+        </is>
+      </c>
+      <c r="G95" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="15" customHeight="1" s="27">
+      <c r="A96" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B96" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C96" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D96" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E96" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h3.csv</t>
+        </is>
+      </c>
+      <c r="F96" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/predicciones_h3.csv</t>
+        </is>
+      </c>
+      <c r="G96" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="15" customHeight="1" s="27">
+      <c r="A97" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B97" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C97" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D97" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E97" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h4.csv</t>
+        </is>
+      </c>
+      <c r="F97" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/predicciones_h4.csv</t>
+        </is>
+      </c>
+      <c r="G97" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="15" customHeight="1" s="27">
+      <c r="A98" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B98" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C98" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D98" s="61" t="inlineStr">
+        <is>
+          <t>resumen</t>
+        </is>
+      </c>
+      <c r="E98" s="61" t="inlineStr">
+        <is>
+          <t>resumen_modeling_horizontes.json</t>
+        </is>
+      </c>
+      <c r="F98" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/resumen_modeling_horizontes.json</t>
+        </is>
+      </c>
+      <c r="G98" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de tamanos y seleccion de features por horizonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="15" customHeight="1" s="27">
+      <c r="A99" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B99" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C99" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D99" s="61" t="inlineStr">
+        <is>
+          <t>tuning</t>
+        </is>
+      </c>
+      <c r="E99" s="61" t="inlineStr">
+        <is>
+          <t>huber_tuning_horizontes.json</t>
+        </is>
+      </c>
+      <c r="F99" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/huber_tuning_horizontes.json</t>
+        </is>
+      </c>
+      <c r="G99" s="61" t="inlineStr">
+        <is>
+          <t>Mejores hiperparametros Huber por fold externo y resumen por horizonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="15" customHeight="1" s="27">
+      <c r="A100" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B100" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C100" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D100" s="61" t="inlineStr">
+        <is>
+          <t>comparacion</t>
+        </is>
+      </c>
+      <c r="E100" s="61" t="inlineStr">
+        <is>
+          <t>comparacion_vs_E1_v5_clean.json</t>
+        </is>
+      </c>
+      <c r="F100" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/comparacion_vs_E1_v5_clean.json</t>
+        </is>
+      </c>
+      <c r="G100" s="61" t="inlineStr">
+        <is>
+          <t>Comparacion de la corrida clean contra E1_v5_clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1" s="27">
+      <c r="A101" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B101" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C101" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D101" s="61" t="inlineStr">
+        <is>
+          <t>comparacion</t>
+        </is>
+      </c>
+      <c r="E101" s="61" t="inlineStr">
+        <is>
+          <t>comparacion_vs_E2_v1_clean.json</t>
+        </is>
+      </c>
+      <c r="F101" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/comparacion_vs_E2_v1_clean.json</t>
+        </is>
+      </c>
+      <c r="G101" s="61" t="inlineStr">
+        <is>
+          <t>Comparacion de la corrida clean contra E2_v1_clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15" customHeight="1" s="27">
+      <c r="A102" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B102" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C102" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D102" s="61" t="inlineStr">
+        <is>
+          <t>metricas</t>
+        </is>
+      </c>
+      <c r="E102" s="61" t="inlineStr">
+        <is>
+          <t>metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="F102" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="G102" s="61" t="inlineStr">
+        <is>
+          <t>Resumen estructurado por horizonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="15" customHeight="1" s="27">
+      <c r="A103" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:10:23</t>
+        </is>
+      </c>
+      <c r="B103" s="61" t="inlineStr">
+        <is>
+          <t>E2_v2_clean</t>
+        </is>
+      </c>
+      <c r="C103" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D103" s="61" t="inlineStr">
+        <is>
+          <t>metadata</t>
+        </is>
+      </c>
+      <c r="E103" s="61" t="inlineStr">
+        <is>
+          <t>metadata_run.json</t>
+        </is>
+      </c>
+      <c r="F103" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v2_clean_20260323_054101/metadata_run.json</t>
+        </is>
+      </c>
+      <c r="G103" s="61" t="inlineStr">
+        <is>
+          <t>Metadata base del run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="15" customHeight="1" s="27">
+      <c r="A104" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B104" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C104" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D104" s="61" t="inlineStr">
+        <is>
+          <t>script_snapshot</t>
+        </is>
+      </c>
+      <c r="E104" s="61" t="inlineStr">
+        <is>
+          <t>run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="F104" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/scripts/run_e2_huber_clean.py</t>
+        </is>
+      </c>
+      <c r="G104" s="61" t="inlineStr">
+        <is>
+          <t>Copia del script ejecutado para reproducibilidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="15" customHeight="1" s="27">
+      <c r="A105" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B105" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C105" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D105" s="61" t="inlineStr">
+        <is>
+          <t>parametros</t>
+        </is>
+      </c>
+      <c r="E105" s="61" t="inlineStr">
+        <is>
+          <t>parametros_run.json</t>
+        </is>
+      </c>
+      <c r="F105" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/parametros_run.json</t>
+        </is>
+      </c>
+      <c r="G105" s="61" t="inlineStr">
+        <is>
+          <t>Parametros del experimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="15" customHeight="1" s="27">
+      <c r="A106" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B106" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C106" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D106" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E106" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h1.csv</t>
+        </is>
+      </c>
+      <c r="F106" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/features_seleccionadas_h1.csv</t>
+        </is>
+      </c>
+      <c r="G106" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="15" customHeight="1" s="27">
+      <c r="A107" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B107" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C107" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D107" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E107" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h2.csv</t>
+        </is>
+      </c>
+      <c r="F107" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/features_seleccionadas_h2.csv</t>
+        </is>
+      </c>
+      <c r="G107" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="15" customHeight="1" s="27">
+      <c r="A108" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B108" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C108" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D108" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E108" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h3.csv</t>
+        </is>
+      </c>
+      <c r="F108" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/features_seleccionadas_h3.csv</t>
+        </is>
+      </c>
+      <c r="G108" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="15" customHeight="1" s="27">
+      <c r="A109" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B109" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C109" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D109" s="61" t="inlineStr">
+        <is>
+          <t>seleccion_features</t>
+        </is>
+      </c>
+      <c r="E109" s="61" t="inlineStr">
+        <is>
+          <t>features_seleccionadas_h4.csv</t>
+        </is>
+      </c>
+      <c r="F109" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/features_seleccionadas_h4.csv</t>
+        </is>
+      </c>
+      <c r="G109" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de combinaciones de features seleccionadas por fold externo. El filtro se calcula solo con el train de cada fold externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="15" customHeight="1" s="27">
+      <c r="A110" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B110" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C110" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D110" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E110" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h1.csv</t>
+        </is>
+      </c>
+      <c r="F110" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/predicciones_h1.csv</t>
+        </is>
+      </c>
+      <c r="G110" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="15" customHeight="1" s="27">
+      <c r="A111" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B111" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C111" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D111" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E111" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h2.csv</t>
+        </is>
+      </c>
+      <c r="F111" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/predicciones_h2.csv</t>
+        </is>
+      </c>
+      <c r="G111" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="15" customHeight="1" s="27">
+      <c r="A112" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B112" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C112" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D112" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E112" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h3.csv</t>
+        </is>
+      </c>
+      <c r="F112" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/predicciones_h3.csv</t>
+        </is>
+      </c>
+      <c r="G112" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="15" customHeight="1" s="27">
+      <c r="A113" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B113" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C113" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D113" s="61" t="inlineStr">
+        <is>
+          <t>predicciones</t>
+        </is>
+      </c>
+      <c r="E113" s="61" t="inlineStr">
+        <is>
+          <t>predicciones_h4.csv</t>
+        </is>
+      </c>
+      <c r="F113" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/predicciones_h4.csv</t>
+        </is>
+      </c>
+      <c r="G113" s="61" t="inlineStr">
+        <is>
+          <t>Predicciones walk-forward para horizonte 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="15" customHeight="1" s="27">
+      <c r="A114" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B114" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C114" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D114" s="61" t="inlineStr">
+        <is>
+          <t>resumen</t>
+        </is>
+      </c>
+      <c r="E114" s="61" t="inlineStr">
+        <is>
+          <t>resumen_modeling_horizontes.json</t>
+        </is>
+      </c>
+      <c r="F114" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/resumen_modeling_horizontes.json</t>
+        </is>
+      </c>
+      <c r="G114" s="61" t="inlineStr">
+        <is>
+          <t>Resumen de tamanos y seleccion de features por horizonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="15" customHeight="1" s="27">
+      <c r="A115" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B115" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C115" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D115" s="61" t="inlineStr">
+        <is>
+          <t>tuning</t>
+        </is>
+      </c>
+      <c r="E115" s="61" t="inlineStr">
+        <is>
+          <t>huber_tuning_horizontes.json</t>
+        </is>
+      </c>
+      <c r="F115" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/huber_tuning_horizontes.json</t>
+        </is>
+      </c>
+      <c r="G115" s="61" t="inlineStr">
+        <is>
+          <t>Mejores hiperparametros Huber por fold externo y resumen por horizonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="15" customHeight="1" s="27">
+      <c r="A116" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B116" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C116" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D116" s="61" t="inlineStr">
+        <is>
+          <t>comparacion</t>
+        </is>
+      </c>
+      <c r="E116" s="61" t="inlineStr">
+        <is>
+          <t>comparacion_vs_E1_v5_clean.json</t>
+        </is>
+      </c>
+      <c r="F116" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/comparacion_vs_E1_v5_clean.json</t>
+        </is>
+      </c>
+      <c r="G116" s="61" t="inlineStr">
+        <is>
+          <t>Comparacion de la corrida clean contra E1_v5_clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="15" customHeight="1" s="27">
+      <c r="A117" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B117" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C117" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D117" s="61" t="inlineStr">
+        <is>
+          <t>comparacion</t>
+        </is>
+      </c>
+      <c r="E117" s="61" t="inlineStr">
+        <is>
+          <t>comparacion_vs_E2_v1_clean.json</t>
+        </is>
+      </c>
+      <c r="F117" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/comparacion_vs_E2_v1_clean.json</t>
+        </is>
+      </c>
+      <c r="G117" s="61" t="inlineStr">
+        <is>
+          <t>Comparacion de la corrida clean contra E2_v1_clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="15" customHeight="1" s="27">
+      <c r="A118" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B118" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C118" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D118" s="61" t="inlineStr">
+        <is>
+          <t>metricas</t>
+        </is>
+      </c>
+      <c r="E118" s="61" t="inlineStr">
+        <is>
+          <t>metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="F118" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/metricas_horizonte.json</t>
+        </is>
+      </c>
+      <c r="G118" s="61" t="inlineStr">
+        <is>
+          <t>Resumen estructurado por horizonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="15" customHeight="1" s="27">
+      <c r="A119" s="61" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:22:49</t>
+        </is>
+      </c>
+      <c r="B119" s="61" t="inlineStr">
+        <is>
+          <t>E2_v3_clean</t>
+        </is>
+      </c>
+      <c r="C119" s="61" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="D119" s="61" t="inlineStr">
+        <is>
+          <t>metadata</t>
+        </is>
+      </c>
+      <c r="E119" s="61" t="inlineStr">
+        <is>
+          <t>metadata_run.json</t>
+        </is>
+      </c>
+      <c r="F119" s="61" t="inlineStr">
+        <is>
+          <t>Experimentos/runs/E2_v3_clean_20260323_061213/metadata_run.json</t>
+        </is>
+      </c>
+      <c r="G119" s="61" t="inlineStr">
+        <is>
+          <t>Metadata base del run.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>